<commit_message>
Resolved Estimates issue of skipping Beverage Service
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/SalesTestData.xlsx
+++ b/src/test/resources/TestData/SalesTestData.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="91">
   <si>
     <t xml:space="preserve">Bill Terms</t>
   </si>
@@ -259,6 +259,12 @@
     <t xml:space="preserve">Work Phone </t>
   </si>
   <si>
+    <t xml:space="preserve">Entrance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery Charges</t>
+  </si>
+  <si>
     <t xml:space="preserve">CaterXpert</t>
   </si>
   <si>
@@ -286,7 +292,7 @@
     <t xml:space="preserve">New York County</t>
   </si>
   <si>
-    <t xml:space="preserve">0</t>
+    <t xml:space="preserve">6</t>
   </si>
   <si>
     <t xml:space="preserve">07:00</t>
@@ -497,112 +503,116 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -861,137 +871,137 @@
   <dimension ref="A1:S2"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="6.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="0" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="15.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="19.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="26.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="16.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="16.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="10.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="15.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="19.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="26.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="16.11"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4"/>
+      <c r="S1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="10" t="n">
+      <c r="I2" s="11" t="n">
         <v>60606</v>
       </c>
-      <c r="J2" s="10" t="n">
+      <c r="J2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="K2" s="10" t="n">
+      <c r="K2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="L2" s="10" t="n">
+      <c r="L2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="10" t="n">
+      <c r="Q2" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="R2" s="10" t="n">
+      <c r="R2" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="S2" s="10"/>
+      <c r="S2" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1012,105 +1022,105 @@
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="6.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="11" t="n">
         <v>12345</v>
       </c>
-      <c r="I2" s="10" t="n">
+      <c r="I2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="J2" s="10" t="n">
+      <c r="J2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="K2" s="10" t="n">
+      <c r="K2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M2" s="10" t="n">
+      <c r="M2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="11" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1133,149 +1143,149 @@
   <dimension ref="A1:X2"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="39.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="6.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="6.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="19.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="15.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="19.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="16.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="26.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="39.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="15.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="19.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="16.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="26.56"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="W1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="X1" s="4"/>
+      <c r="X1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="10" t="n">
+      <c r="K2" s="11" t="n">
         <v>60606</v>
       </c>
-      <c r="L2" s="10" t="n">
+      <c r="L2" s="11" t="n">
         <v>7417417411</v>
       </c>
-      <c r="M2" s="10" t="n">
+      <c r="M2" s="11" t="n">
         <v>7417417411</v>
       </c>
-      <c r="N2" s="10" t="n">
+      <c r="N2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="0" t="s">
+      <c r="O2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="P2" s="10" t="n">
+      <c r="P2" s="11" t="n">
         <v>8528528522</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="Q2" s="11" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1295,215 +1305,236 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA19"/>
+  <dimension ref="A1:AD19"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="18.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="18.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="13.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="16.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="17.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="14.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16377" style="0" width="11.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="15.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="18.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="18" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="13.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="14.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="11.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="19.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="23.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16377" style="1" width="11.56"/>
   </cols>
   <sheetData>
-    <row r="1" s="13" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+    <row r="1" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="U1" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="V1" s="14" t="s">
+      <c r="V1" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="W1" s="13" t="s">
+      <c r="W1" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="X1" s="13" t="s">
+      <c r="X1" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="Y1" s="15" t="s">
+      <c r="Y1" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="Z1" s="15" t="s">
+      <c r="Z1" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="AA1" s="13" t="s">
+      <c r="AA1" s="14" t="s">
         <v>77</v>
+      </c>
+      <c r="AB1" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC1" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD1" s="14" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="B2" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="17" t="s">
+      <c r="C2" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="H2" s="17" t="n">
+      <c r="E2" s="17"/>
+      <c r="F2" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="17" t="n">
+      <c r="J2" s="18" t="n">
         <v>150</v>
       </c>
-      <c r="K2" s="17" t="n">
+      <c r="K2" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L2" s="17" t="n">
+      <c r="L2" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="M2" s="17" t="n">
+      <c r="M2" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="N2" s="17" t="n">
+      <c r="N2" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="P2" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q2" s="17" t="s">
+      <c r="O2" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="R2" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="19" t="s">
+      <c r="P2" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="T2" s="17" t="n">
+      <c r="Q2" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="R2" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="S2" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="T2" s="18" t="n">
         <v>8528528522</v>
       </c>
-      <c r="U2" s="17" t="s">
+      <c r="U2" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="17" t="n">
+      <c r="V2" s="18" t="n">
         <v>7417417411</v>
       </c>
-      <c r="W2" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="X2" s="20" t="n">
+      <c r="W2" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="X2" s="21" t="n">
         <v>0.458333333333333</v>
       </c>
-      <c r="Y2" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z2" s="0" t="n">
+      <c r="Y2" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AA2" s="0" t="n">
+      <c r="AA2" s="1" t="n">
         <v>9639639633</v>
+      </c>
+      <c r="AB2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD2" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P5" s="22"/>
+      <c r="P5" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="S7" s="23"/>
+      <c r="S7" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="S9" s="24"/>
+      <c r="S9" s="25"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="T11" s="25"/>
+      <c r="T11" s="26"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="T19" s="26"/>
+      <c r="T19" s="27"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Commiting stable code to git
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/SalesTestData.xlsx
+++ b/src/test/resources/TestData/SalesTestData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Create Customer" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="94">
   <si>
     <t xml:space="preserve">Bill Terms</t>
   </si>
@@ -82,13 +82,13 @@
     <t xml:space="preserve">New</t>
   </si>
   <si>
-    <t xml:space="preserve">Jared clark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jared </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jared</t>
+    <t xml:space="preserve">Coleman Darius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coleman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darius</t>
   </si>
   <si>
     <t xml:space="preserve">Building</t>
@@ -115,6 +115,9 @@
     <t xml:space="preserve">Last Name</t>
   </si>
   <si>
+    <t xml:space="preserve">Middle Initial</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dear Name</t>
   </si>
   <si>
@@ -265,6 +268,9 @@
     <t xml:space="preserve">Delivery Charges</t>
   </si>
   <si>
+    <t xml:space="preserve">Comments</t>
+  </si>
+  <si>
     <t xml:space="preserve">CaterXpert</t>
   </si>
   <si>
@@ -296,6 +302,9 @@
   </si>
   <si>
     <t xml:space="preserve">07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event Comments</t>
   </si>
 </sst>
 </file>
@@ -307,7 +316,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,14 +370,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
@@ -503,7 +504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -541,34 +542,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -576,30 +577,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -608,7 +605,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -956,37 +953,37 @@
       <c r="C2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>21</v>
+      <c r="D2" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="11" t="n">
+      <c r="I2" s="10" t="n">
         <v>60606</v>
       </c>
-      <c r="J2" s="11" t="n">
+      <c r="J2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="K2" s="11" t="n">
+      <c r="K2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="L2" s="11" t="n">
+      <c r="L2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="N2" s="10" t="s">
         <v>26</v>
       </c>
       <c r="O2" s="8" t="s">
@@ -995,13 +992,13 @@
       <c r="P2" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="11" t="n">
+      <c r="Q2" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="R2" s="11" t="n">
+      <c r="R2" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="S2" s="11"/>
+      <c r="S2" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1019,21 +1016,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="12.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="12.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="12.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1050,77 +1047,83 @@
         <v>31</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>33</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>35</v>
       </c>
       <c r="N1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="F2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="G2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="H2" s="11" t="n">
+      <c r="H2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="10" t="n">
         <v>12345</v>
       </c>
-      <c r="I2" s="11" t="n">
+      <c r="J2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="J2" s="11" t="n">
+      <c r="K2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="K2" s="11" t="n">
+      <c r="L2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" s="11" t="n">
+      <c r="M2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="O2" s="10" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1168,23 +1171,23 @@
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="12" t="s">
+      <c r="A1" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>5</v>
@@ -1196,7 +1199,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>8</v>
@@ -1223,7 +1226,7 @@
         <v>15</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>16</v>
@@ -1232,60 +1235,60 @@
         <v>17</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="X1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K2" s="11" t="n">
+      <c r="J2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="10" t="n">
         <v>60606</v>
       </c>
-      <c r="L2" s="11" t="n">
+      <c r="L2" s="10" t="n">
         <v>7417417411</v>
       </c>
-      <c r="M2" s="11" t="n">
+      <c r="M2" s="10" t="n">
         <v>7417417411</v>
       </c>
-      <c r="N2" s="11" t="n">
+      <c r="N2" s="10" t="n">
         <v>1</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P2" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="P2" s="10" t="n">
         <v>8528528522</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="10" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1305,7 +1308,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -1333,177 +1336,181 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="12.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="17.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="14.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="11.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="19.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="0" width="23.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="11.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="19.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="23.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16377" style="1" width="11.56"/>
   </cols>
   <sheetData>
-    <row r="1" s="14" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="14" t="s">
+    <row r="1" s="13" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>54</v>
       </c>
+      <c r="B1" s="13" t="s">
+        <v>55</v>
+      </c>
       <c r="C1" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="G1" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="I1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="J1" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="K1" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="M1" s="14" t="s">
+      <c r="L1" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="M1" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="N1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="O1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="Q1" s="14" t="s">
+      <c r="P1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="R1" s="14" t="s">
+      <c r="Q1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="S1" s="14" t="s">
+      <c r="R1" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="T1" s="14" t="s">
+      <c r="S1" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="T1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="V1" s="15" t="s">
+      <c r="U1" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="W1" s="14" t="s">
+      <c r="V1" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="X1" s="14" t="s">
+      <c r="W1" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="Y1" s="16" t="s">
+      <c r="X1" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="Z1" s="16" t="s">
+      <c r="Y1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="AA1" s="14" t="s">
+      <c r="Z1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="AB1" s="14" t="s">
+      <c r="AA1" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="AC1" s="14" t="s">
+      <c r="AB1" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="AD1" s="14" t="s">
+      <c r="AC1" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD1" s="13" t="s">
         <v>17</v>
+      </c>
+      <c r="AE1" s="13" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>81</v>
+        <v>82</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>83</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="D2" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="H2" s="18" t="n">
+      <c r="E2" s="16"/>
+      <c r="F2" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" s="17" t="n">
         <v>20</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="J2" s="17" t="n">
         <v>150</v>
       </c>
-      <c r="K2" s="18" t="n">
+      <c r="K2" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="L2" s="18" t="n">
+      <c r="L2" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="M2" s="18" t="n">
+      <c r="M2" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="N2" s="18" t="n">
+      <c r="N2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="P2" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q2" s="18" t="s">
+      <c r="O2" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="R2" s="18" t="n">
+      <c r="P2" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q2" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="R2" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="S2" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="T2" s="18" t="n">
+      <c r="S2" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="T2" s="17" t="n">
         <v>8528528522</v>
       </c>
-      <c r="U2" s="18" t="s">
+      <c r="U2" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="18" t="n">
+      <c r="V2" s="17" t="n">
         <v>7417417411</v>
       </c>
-      <c r="W2" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="X2" s="21" t="n">
+      <c r="W2" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="X2" s="20" t="n">
         <v>0.458333333333333</v>
       </c>
-      <c r="Y2" s="22" t="s">
-        <v>82</v>
+      <c r="Y2" s="21" t="s">
+        <v>84</v>
       </c>
       <c r="Z2" s="1" t="n">
         <v>10</v>
@@ -1517,24 +1524,27 @@
       <c r="AC2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="AD2" s="0" t="n">
+      <c r="AD2" s="1" t="n">
         <v>10</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P5" s="23"/>
+      <c r="P5" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="S7" s="24"/>
+      <c r="S7" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="S9" s="25"/>
+      <c r="S9" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="T11" s="26"/>
+      <c r="T11" s="25"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="T19" s="27"/>
+      <c r="T19" s="26"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Started Regression Test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/SalesTestData.xlsx
+++ b/src/test/resources/TestData/SalesTestData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Create Customer" sheetId="1" state="visible" r:id="rId3"/>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">New</t>
   </si>
   <si>
-    <t xml:space="preserve">Parkar  Darius</t>
+    <t xml:space="preserve">Peter Hudson</t>
   </si>
   <si>
     <t xml:space="preserve">Nora</t>
@@ -322,10 +322,10 @@
     <t xml:space="preserve">New York County</t>
   </si>
   <si>
-    <t xml:space="preserve">10,07:00 PM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11,10:00 PM</t>
+    <t xml:space="preserve">1,07:00 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,10:00 PM</t>
   </si>
   <si>
     <t xml:space="preserve">Event Comments</t>

</xml_diff>

<commit_message>
Added Create Event and  Menu Service to Regression Tests
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/SalesTestData.xlsx
+++ b/src/test/resources/TestData/SalesTestData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Create Customer" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="103">
   <si>
     <t xml:space="preserve">Bill Terms</t>
   </si>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">New</t>
   </si>
   <si>
-    <t xml:space="preserve">Peter Hudson</t>
+    <t xml:space="preserve">Peter Nolan</t>
   </si>
   <si>
     <t xml:space="preserve">Nora</t>
@@ -166,151 +166,154 @@
     <t xml:space="preserve">Daniel</t>
   </si>
   <si>
-    <t xml:space="preserve">Grace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parkar</t>
+    <t xml:space="preserve">Peter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nolan</t>
   </si>
   <si>
     <t xml:space="preserve">illions</t>
   </si>
   <si>
+    <t xml:space="preserve">peter.nolan@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grace Broad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer/Potential Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer/Potential Customer Types </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact First Name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact Last Name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referral Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business Units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ecatering Business Unit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jonas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 N Lasalle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Studtmann, Jenna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">demo@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EventType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PropasalStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EventTheam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adult Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PerPersonCost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kidsCount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StaffGuests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BandGuests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MiscCount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue Stream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">County</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Begin Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated $/Person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work Phone </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery Charges</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CaterXpert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Day Catering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With Client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Social</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wedding</t>
+  </si>
+  <si>
     <t xml:space="preserve">Broad@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grace Broad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer/Potential Customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer/Potential Customer Types </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact First Name </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact Last Name </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referral Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Business Units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ecatering Business Unit </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jonas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 N Lasalle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Studtmann, Jenna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">demo@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EventType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PropasalStatus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EventTheam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Event Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adult Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PerPersonCost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kidsCount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">StaffGuests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BandGuests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MiscCount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Event Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revenue Stream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">County</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Begin Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">City</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work Phone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated $/Person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work Phone </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delivery Charges</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CaterXpert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Day Catering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">With Client</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wedding</t>
   </si>
   <si>
     <t xml:space="preserve">Walker , Jack</t>
@@ -1547,7 +1550,7 @@
         <v>20</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="J2" s="18" t="n">
         <v>150</v>
@@ -1565,19 +1568,19 @@
         <v>1</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P2" s="18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="R2" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S2" s="21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="T2" s="18" t="n">
         <v>8528528522</v>
@@ -1607,7 +1610,7 @@
         <v>10</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>